<commit_message>
Begining CD code development for CD
</commit_message>
<xml_diff>
--- a/EuroferExperiments/input/input_parameters.xlsx
+++ b/EuroferExperiments/input/input_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fuqih\Documents\RadiationDamage\EuroferMicro\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\Repos\EuroferMicrostructure\EuroferExperiments\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9040D5B-7F91-4B9B-941B-C47A79A88306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7FD243-E6C8-471C-929D-4B45645B3606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Material_Environment" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="187">
   <si>
     <t>Notation</t>
   </si>
@@ -481,9 +481,6 @@
     <t>binding energy of a triinterstitial</t>
   </si>
   <si>
-    <t>mu</t>
-  </si>
-  <si>
     <t>shear modulus</t>
   </si>
   <si>
@@ -514,21 +511,6 @@
     <t>E_m_2i</t>
   </si>
   <si>
-    <t>D_i_0</t>
-  </si>
-  <si>
-    <t>m^2/s</t>
-  </si>
-  <si>
-    <t>interstitial diffusion pre-factor</t>
-  </si>
-  <si>
-    <t>D_v_0</t>
-  </si>
-  <si>
-    <t>vacancy diffusion prefactor</t>
-  </si>
-  <si>
     <t>recom</t>
   </si>
   <si>
@@ -575,6 +557,45 @@
   </si>
   <si>
     <t>Collision cascade efficiency to generate a void</t>
+  </si>
+  <si>
+    <t>nu_h</t>
+  </si>
+  <si>
+    <t>helium attempt frequency</t>
+  </si>
+  <si>
+    <t>E_m_h</t>
+  </si>
+  <si>
+    <t>helium migration barrier</t>
+  </si>
+  <si>
+    <t>b_r</t>
+  </si>
+  <si>
+    <t>resolution parameter</t>
+  </si>
+  <si>
+    <t>mu_s</t>
+  </si>
+  <si>
+    <t>B_2</t>
+  </si>
+  <si>
+    <t>B_3</t>
+  </si>
+  <si>
+    <t>m^3/atom</t>
+  </si>
+  <si>
+    <t>m^6/atom^2</t>
+  </si>
+  <si>
+    <t>second virial coefficient for helium</t>
+  </si>
+  <si>
+    <t>third virial coefficient for helium</t>
   </si>
 </sst>
 </file>
@@ -963,7 +984,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="49" customWidth="1"/>
@@ -972,7 +993,7 @@
     <col min="5" max="5" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -989,7 +1010,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1006,7 +1027,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1023,7 +1044,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -1040,7 +1061,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1057,7 +1078,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1074,7 +1095,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -1085,13 +1106,13 @@
         <v>25</v>
       </c>
       <c r="D7" s="2">
-        <v>1E-3</v>
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="E7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -1108,7 +1129,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -1125,7 +1146,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>139</v>
       </c>
@@ -1142,7 +1163,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>141</v>
       </c>
@@ -1166,18 +1187,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F36"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="37" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1194,7 +1215,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -1211,12 +1232,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="B3" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C3" t="s">
         <v>11</v>
@@ -1225,15 +1246,15 @@
         <v>2.4800000000000002E-10</v>
       </c>
       <c r="E3" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B4" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
@@ -1242,10 +1263,10 @@
         <v>1.43E-10</v>
       </c>
       <c r="E4" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>64</v>
       </c>
@@ -1262,7 +1283,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>68</v>
       </c>
@@ -1279,19 +1300,19 @@
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="B7" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="D7" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -1302,30 +1323,30 @@
         <v>39</v>
       </c>
       <c r="D9">
-        <v>0.85</v>
+        <v>0.34</v>
       </c>
       <c r="E9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B10" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C10" t="s">
         <v>39</v>
       </c>
       <c r="D10">
-        <v>0.75</v>
+        <v>0.2</v>
       </c>
       <c r="E10" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -1336,304 +1357,344 @@
         <v>39</v>
       </c>
       <c r="D11">
-        <v>1.1499999999999999</v>
+        <v>0.6</v>
       </c>
       <c r="E11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>44</v>
-      </c>
-      <c r="B12" t="s">
-        <v>45</v>
+        <v>176</v>
       </c>
       <c r="C12" t="s">
         <v>39</v>
       </c>
       <c r="D12">
-        <v>1.6</v>
+        <v>0.08</v>
       </c>
       <c r="E12" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
         <v>39</v>
       </c>
       <c r="D13">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="E13" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>144</v>
+        <v>47</v>
       </c>
       <c r="B14" t="s">
-        <v>145</v>
+        <v>48</v>
       </c>
       <c r="C14" t="s">
         <v>39</v>
       </c>
       <c r="D14">
-        <v>1.42</v>
+        <v>4</v>
       </c>
       <c r="E14" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>144</v>
+      </c>
+      <c r="B15" t="s">
         <v>145</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>146</v>
-      </c>
-      <c r="B15" t="s">
-        <v>147</v>
       </c>
       <c r="C15" t="s">
         <v>39</v>
       </c>
       <c r="D15">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="E15" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="16" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>146</v>
+      </c>
+      <c r="B16" t="s">
+        <v>147</v>
+      </c>
+      <c r="C16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16">
+        <v>2</v>
+      </c>
+      <c r="E16" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>50</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>51</v>
-      </c>
-      <c r="C17" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" s="2">
-        <v>1.37E+19</v>
-      </c>
-      <c r="E17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>54</v>
-      </c>
-      <c r="B18" t="s">
-        <v>55</v>
       </c>
       <c r="C18" t="s">
         <v>52</v>
       </c>
       <c r="D18" s="2">
-        <v>1.25E+18</v>
+        <f>2.4*6240000000000000000</f>
+        <v>1.4976E+19</v>
       </c>
       <c r="E18" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" s="2">
+        <f>0.6*6240000000000000000</f>
+        <v>3.744E+18</v>
+      </c>
+      <c r="E19" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D19" s="8"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D20" s="8"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>57</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B21" t="s">
         <v>58</v>
-      </c>
-      <c r="C20" t="s">
-        <v>59</v>
-      </c>
-      <c r="D20" s="2">
-        <f>D6*D33/(D2)^2</f>
-        <v>480504670155.01984</v>
-      </c>
-      <c r="E20" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>61</v>
-      </c>
-      <c r="B21" t="s">
-        <v>62</v>
       </c>
       <c r="C21" t="s">
         <v>59</v>
       </c>
       <c r="D21" s="2">
-        <f>D6*D34/(D2)^2</f>
-        <v>291294439.8259083</v>
+        <v>4000000000000</v>
       </c>
       <c r="E21" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" t="s">
+        <v>62</v>
+      </c>
+      <c r="C22" t="s">
+        <v>59</v>
+      </c>
+      <c r="D22" s="2">
+        <v>40000000000000</v>
+      </c>
+      <c r="E22" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="22" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
+        <v>174</v>
+      </c>
+      <c r="C23" t="s">
+        <v>59</v>
+      </c>
+      <c r="D23" s="2">
+        <v>2000000000000</v>
+      </c>
+      <c r="E23" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>178</v>
+      </c>
+      <c r="D24" s="2">
+        <v>1</v>
+      </c>
+      <c r="E24" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>72</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B26" t="s">
         <v>73</v>
       </c>
-      <c r="C23" t="s">
-        <v>70</v>
-      </c>
-      <c r="D23" s="2">
+      <c r="C26" t="s">
+        <v>70</v>
+      </c>
+      <c r="D26" s="2">
         <v>0.01</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E26" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>177</v>
-      </c>
-      <c r="B24" t="s">
-        <v>179</v>
-      </c>
-      <c r="C24" t="s">
-        <v>70</v>
-      </c>
-      <c r="D24" s="2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>171</v>
+      </c>
+      <c r="B27" t="s">
+        <v>173</v>
+      </c>
+      <c r="C27" t="s">
+        <v>70</v>
+      </c>
+      <c r="D27" s="2">
         <v>0.01</v>
       </c>
-      <c r="E24" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="E27" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>75</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B28" t="s">
         <v>76</v>
       </c>
-      <c r="C25" t="s">
-        <v>70</v>
-      </c>
-      <c r="D25" s="2">
+      <c r="C28" t="s">
+        <v>70</v>
+      </c>
+      <c r="D28" s="2">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E28" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>78</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B29" t="s">
         <v>79</v>
       </c>
-      <c r="C26" t="s">
-        <v>70</v>
-      </c>
-      <c r="D26" s="2">
-        <f>D25</f>
+      <c r="C29" t="s">
+        <v>70</v>
+      </c>
+      <c r="D29" s="2">
+        <f>D28</f>
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E29" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="27" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="30" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>81</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B31" t="s">
         <v>82</v>
       </c>
-      <c r="C28" t="s">
-        <v>70</v>
-      </c>
-      <c r="D28">
+      <c r="C31" t="s">
+        <v>70</v>
+      </c>
+      <c r="D31">
         <v>2</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E31" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>180</v>
+      </c>
+      <c r="B32" t="s">
         <v>148</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C32" t="s">
+        <v>137</v>
+      </c>
+      <c r="D32" s="2">
+        <v>80000000000</v>
+      </c>
+      <c r="E32" t="s">
+        <v>148</v>
+      </c>
+      <c r="F32" s="2"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>149</v>
       </c>
-      <c r="C29" t="s">
-        <v>137</v>
-      </c>
-      <c r="D29" s="2">
-        <v>30000000000</v>
-      </c>
-      <c r="E29" t="s">
-        <v>149</v>
-      </c>
-      <c r="F29" s="2"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="B33" t="s">
         <v>150</v>
       </c>
-      <c r="B30" t="s">
-        <v>151</v>
-      </c>
-      <c r="C30" t="s">
-        <v>70</v>
-      </c>
-      <c r="D30" s="2">
+      <c r="C33" t="s">
+        <v>70</v>
+      </c>
+      <c r="D33" s="2">
         <v>0.34</v>
       </c>
-      <c r="E30" t="s">
-        <v>151</v>
-      </c>
-      <c r="F30" s="2"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>159</v>
-      </c>
-      <c r="B33" t="s">
-        <v>161</v>
-      </c>
-      <c r="C33" t="s">
-        <v>160</v>
-      </c>
-      <c r="D33" s="2">
-        <v>8.1881999999999997E-10</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>162</v>
-      </c>
-      <c r="B34" t="s">
-        <v>163</v>
-      </c>
-      <c r="C34" t="s">
-        <v>160</v>
-      </c>
-      <c r="D34" s="2">
-        <v>4.9638999999999997E-13</v>
+      <c r="E33" t="s">
+        <v>150</v>
+      </c>
+      <c r="F33" s="2"/>
+    </row>
+    <row r="34" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>181</v>
+      </c>
+      <c r="C35" t="s">
+        <v>183</v>
+      </c>
+      <c r="D35" s="2">
+        <v>1.5700000000000001E-29</v>
+      </c>
+      <c r="E35" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>182</v>
+      </c>
+      <c r="C36" t="s">
+        <v>184</v>
+      </c>
+      <c r="D36" s="2">
+        <v>1.8399999999999998E-58</v>
+      </c>
+      <c r="E36" t="s">
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -1645,16 +1706,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="7" customWidth="1"/>
-    <col min="4" max="4" width="11.28515625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="11.26953125" style="4" customWidth="1"/>
     <col min="5" max="5" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1671,9 +1732,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B2" t="s">
         <v>84</v>
@@ -1688,9 +1749,9 @@
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B3" t="s">
         <v>86</v>
@@ -1705,9 +1766,9 @@
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B4" t="s">
         <v>88</v>
@@ -1722,7 +1783,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>90</v>
       </c>
@@ -1739,7 +1800,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>93</v>
       </c>
@@ -1756,7 +1817,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1773,10 +1834,10 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="D8" s="6"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>99</v>
       </c>
@@ -1793,7 +1854,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>103</v>
       </c>
@@ -1810,12 +1871,12 @@
         <v>105</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>151</v>
+      </c>
+      <c r="B11" t="s">
         <v>152</v>
-      </c>
-      <c r="B11" t="s">
-        <v>153</v>
       </c>
       <c r="C11" t="s">
         <v>11</v>
@@ -1824,15 +1885,15 @@
         <v>2.4999999999999999E-8</v>
       </c>
       <c r="E11" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>11</v>
@@ -1841,13 +1902,13 @@
         <v>2.4999999999999999E-8</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="D13" s="6"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>106</v>
       </c>
@@ -1864,7 +1925,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>109</v>
       </c>
@@ -1881,7 +1942,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>112</v>
       </c>
@@ -1898,7 +1959,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>115</v>
       </c>
@@ -1915,7 +1976,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>118</v>
       </c>
@@ -1932,7 +1993,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>121</v>
       </c>
@@ -1949,7 +2010,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>124</v>
       </c>
@@ -1966,10 +2027,10 @@
         <v>126</v>
       </c>
     </row>
-    <row r="21" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="D21" s="6"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>11</v>
       </c>
@@ -1986,7 +2047,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>101</v>
       </c>
@@ -2003,7 +2064,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>131</v>
       </c>
@@ -2020,7 +2081,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>134</v>
       </c>

</xml_diff>